<commit_message>
thêm ràng buộc giáo viên dại các môn liên quan tới ngành vào
</commit_message>
<xml_diff>
--- a/docs/samples/school_demo_small.xlsx
+++ b/docs/samples/school_demo_small.xlsx
@@ -707,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -721,6 +721,11 @@
           <t>name</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -733,6 +738,11 @@
           <t>GV1</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -745,6 +755,11 @@
           <t>GV2</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -757,6 +772,11 @@
           <t>GV3</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -769,6 +789,11 @@
           <t>GV4</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -781,6 +806,11 @@
           <t>GV5</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -793,6 +823,11 @@
           <t>GV6</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -805,6 +840,11 @@
           <t>GV7</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -817,6 +857,11 @@
           <t>GV8</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -829,6 +874,11 @@
           <t>GV9</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -841,6 +891,11 @@
           <t>GV10</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -853,6 +908,11 @@
           <t>GV11</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -865,6 +925,11 @@
           <t>GV12</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -877,6 +942,11 @@
           <t>GV13</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -889,6 +959,11 @@
           <t>GV14</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -901,6 +976,11 @@
           <t>GV15</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -913,6 +993,11 @@
           <t>GV16</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -925,6 +1010,11 @@
           <t>GV17</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -937,6 +1027,11 @@
           <t>GV18</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -949,6 +1044,11 @@
           <t>GV19</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -959,6 +1059,11 @@
       <c r="B21" t="inlineStr">
         <is>
           <t>GV20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>English</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1163,6 +1268,11 @@
           <t>required_room_type</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1182,7 +1292,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GV10</t>
+          <t>GV1</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1193,6 +1303,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1212,7 +1327,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GV17</t>
+          <t>GV2</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1223,6 +1338,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1242,7 +1362,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GV18</t>
+          <t>GV3</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1253,6 +1373,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1272,7 +1397,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GV19</t>
+          <t>GV4</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1283,6 +1408,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1302,7 +1432,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>GV2</t>
+          <t>GV18</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1313,6 +1443,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1332,7 +1467,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GV6</t>
+          <t>GV19</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1343,6 +1478,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1362,7 +1502,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GV20</t>
+          <t>GV9</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1373,6 +1513,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1392,7 +1537,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GV3</t>
+          <t>GV10</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1403,6 +1548,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1422,7 +1572,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GV4</t>
+          <t>GV6</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1433,6 +1583,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1452,7 +1607,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GV5</t>
+          <t>GV7</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1463,6 +1618,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1482,7 +1642,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>GV11</t>
+          <t>GV16</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1493,6 +1653,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1512,7 +1677,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GV7</t>
+          <t>GV18</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1523,6 +1688,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1542,7 +1712,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GV6</t>
+          <t>GV9</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1553,6 +1723,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1572,7 +1747,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GV12</t>
+          <t>GV10</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1583,6 +1758,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1602,7 +1782,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GV7</t>
+          <t>GV8</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1613,6 +1793,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1632,7 +1817,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>GV8</t>
+          <t>GV6</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1643,6 +1828,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1662,7 +1852,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>GV9</t>
+          <t>GV19</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1673,6 +1863,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1692,7 +1887,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GV10</t>
+          <t>GV20</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1703,6 +1898,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1722,7 +1922,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GV13</t>
+          <t>GV6</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1733,6 +1933,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1752,7 +1957,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GV17</t>
+          <t>GV9</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1763,6 +1968,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1782,7 +1992,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GV18</t>
+          <t>GV10</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1793,6 +2003,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1812,7 +2027,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GV19</t>
+          <t>GV7</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1823,6 +2038,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1842,7 +2062,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GV2</t>
+          <t>GV20</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1853,6 +2073,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1872,7 +2097,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GV8</t>
+          <t>GV16</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1883,6 +2108,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1902,7 +2132,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GV14</t>
+          <t>GV7</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1913,6 +2143,11 @@
           <t>mba</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1932,7 +2167,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GV15</t>
+          <t>GV8</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1943,6 +2178,11 @@
           <t>mba</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1962,7 +2202,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GV20</t>
+          <t>GV9</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1973,6 +2213,11 @@
           <t>mba</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1992,7 +2237,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GV3</t>
+          <t>GV10</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2003,6 +2248,11 @@
           <t>mba</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2022,7 +2272,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GV1</t>
+          <t>GV11</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2033,6 +2283,11 @@
           <t>art</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2052,7 +2307,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>GV4</t>
+          <t>GV12</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2063,6 +2318,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2082,7 +2342,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GV5</t>
+          <t>GV13</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2093,6 +2353,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2112,7 +2377,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>GV16</t>
+          <t>GV17</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2123,6 +2388,11 @@
           <t>standard</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2142,7 +2412,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>GV9</t>
+          <t>GV18</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2151,6 +2421,11 @@
       <c r="F34" t="inlineStr">
         <is>
           <t>standard</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>English</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2231,31 +2506,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sức chứa</t>
+          <t>Nhóm chuyên môn</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tạm đặt 30 cho mọi phòng, chờ số chính xác.</t>
+          <t>Cột department: giáo viên chỉ dạy môn cùng nhóm (IT, Business, Design, English).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>G311 (loại khỏi bài toán)</t>
+          <t>Sức chứa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hội trường, tổ chức sự kiện</t>
+          <t>Tạm đặt 30 cho mọi phòng, chờ số chính xác.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>G312 (loại khỏi bài toán)</t>
+          <t>G311 (loại khỏi bài toán)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2267,70 +2542,82 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G315 (loại khỏi bài toán)</t>
+          <t>G312 (loại khỏi bài toán)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Phòng tư vấn tuyển sinh</t>
+          <t>Hội trường, tổ chức sự kiện</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>G320 (loại khỏi bài toán)</t>
+          <t>G315 (loại khỏi bài toán)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Phòng để đồ, chưa có thông tin</t>
+          <t>Phòng tư vấn tuyển sinh</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>G501 (loại khỏi bài toán)</t>
+          <t>G320 (loại khỏi bài toán)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Phòng Director</t>
+          <t>Phòng để đồ, chưa có thông tin</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>G505 (loại khỏi bài toán)</t>
+          <t>G501 (loại khỏi bài toán)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Academic Affairs Administration Dept.</t>
+          <t>Phòng Director</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>G506 (loại khỏi bài toán)</t>
+          <t>G505 (loại khỏi bài toán)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Thư viện</t>
+          <t>Academic Affairs Administration Dept.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>G506 (loại khỏi bài toán)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Thư viện</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>G507 (loại khỏi bài toán)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Student service</t>
         </is>

</xml_diff>